<commit_message>
successfully create  and debugging tas code
</commit_message>
<xml_diff>
--- a/src/scrapers/output_scrape/tas/requirements_tas.xlsx
+++ b/src/scrapers/output_scrape/tas/requirements_tas.xlsx
@@ -1422,11 +1422,120 @@
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>[Minimum Requirements]
--
+You must have established and operated a business in Tasmania for at least 12 months. The business must be solely owned or co-owned with your spouse.
+Your business must still have been in profit after paying yourself a salary of at least 85 per cent of the Temporary Skilled Migration Income Threshold (currently $65,037)*. This income must come from genuine business activity and not be significantly supplemented by non-business sources such as personal savings, loans from family, or other external financial support.
+You must demonstrate awareness of fair employment practices by completing key units from the Fair Work Ombudsman's online learning centre.
+Owners of massage therapy businesses must have a related skills assessment and a verifiable health fund provider number.
+Subcontractors and independent contractors are not eligible under this pathway (refer to Tasmanian Skilled Employment or Tasmanian Established Resident pathways.
 [Priority Attributes]
--
+The following attributes are used to rank Registrations of Interest. Only the most competitive candidates are invited to apply for nomination. There are no Gold or Green priority attributes for the Tasmanian Business Operator pathway. Candidates with at least one orange-plus priority attribute are considered a high priority and will be the first Orange pass candidates invited to apply for nomination. ORANGE PLUS Points You have received a personal income from your business for over 12 months of at least $102,956 per year or $38.72 per hour and your business is still in profit. 40 Your business had a turnover of more than $500,000 in the last financial year. 25 Your business employs more than 10 local Australian citizens or permanent residents or provisional visa holders. 25
+The following attributes are used to rank Registrations of Interest. Only the most competitive candidates are invited to apply for nomination.
+There are no Gold or Green priority attributes for the Tasmanian Business Operator pathway.
+Candidates with at least one orange-plus priority attribute are considered a high priority and will be the first Orange pass candidates invited to apply for nomination.
+ORANGE PLUS
+Points
+You have received a personal income from your business for over 12 months of at least $102,956 per year or $38.72 per hour and your business is still in profit.
+income from your business
+40
+Your business had a turnover of more than $500,000 in the last financial year.
+Your business
+25
+Your business employs more than 10 local Australian citizens or permanent residents or provisional visa holders.
+ORANGE Points You have a skills assessment which is directly related to your current business operation. 12 You received personal earnings from your business of more than $76,515, but less than $102,956 in the last year, and your business is still in profit. 12 You received earnings from your business of more than $68,863 but less than $76,515 in the last year, and your business is still in profit. 10 You hold a qualification that is directly relevant to your current business activities (at least Certificate III), excluding online courses or qualifications obtained through Recognition of Prior Learning. 5 Your spouse has been employed in Tasmania for the past six months in a role that paid at least $ 57,000 per year, or a base hourly rate of $28.85 . 4 You have operated your business in Tasmania for more than 18 consecutive months. 3 You employ at least 3 full time employees who are Australian citizens or permanent residents or provisional visa holders 3 You have resided in Tasmania continuously for three years or more. 3 You have Proficient / Superior English , or you have an exemption to the English language requirements based on your passport country. 2 You have resided in Tasmania continuously for two years but less than three years. 2
+ORANGE
+You have a skills assessment which is directly related to your current business operation.
+directly related
+12
+You received personal earnings from your business of more than $76,515, but less than $102,956 in the last year, and your business is still in profit.
+earnings from your business
+You received earnings from your business of more than $68,863 but less than $76,515 in the last year, and your business is still in profit.
+10
+You hold a qualification that is directly relevant to your current business activities (at least Certificate III), excluding online courses or qualifications obtained through Recognition of Prior Learning.
+5
+Your spouse has been employed in Tasmania for the past six months in a role that paid at least $ 57,000 per year, or a base hourly rate of $28.85 .
+57,000 per year, or a base hourly rate of $28.85
+4
+You have operated your business in Tasmania for more than 18 consecutive months.
+operated your business
+3
+You employ at least 3 full time employees who are Australian citizens or permanent residents or provisional visa holders
+You have resided in Tasmania continuously for three years or more.
+You have Proficient / Superior English , or you have an exemption to the English language requirements based on your passport country.
+Proficient / Superior English
+exemption
+2
+You have resided in Tasmania continuously for two years but less than three years.
 [Required Documents]
--</t>
+Migration Tasmania may request additional documents or information. People or organisations listed in the application, including education providers, employers and real estate agents, may also be contacted to confirm the information you provide.
+After lodging the application, you can submit additional documents until the application has been assigned to a case officer, or after a case officer requests further information.
+All information you provide must be current, true and correct.
+Where documentation or information is found to be false or misleading, the application will be declined, and details are likely to be passed on to other relevant agencies such as the Department of Home Affairs.
+Skills assessments and English tests must be current at time of nomination. If they are not, the Department of Home Affairs may refuse the visa application.
+Passport (Bio-Data page).
+SkillSelect Expression of Interest (EOI) including the personal, educational or employment details referred to in the Registration of Interest and nomination application.
+Skills assessment issued by the relevant assessing body for your stated occupation. Must be dated within the last three years.
+English language report ( English proficiency test result ) dated within the last three years. If you hold a passport issued by the United Kingdom, Canada, New Zealand, United States of America, or Republic of Ireland and do not need to complete an English language test for your skilled visa please attach a copy of your passport bio data page.
+Curriculum vitae (CV)/resume which includes all study and employment from the last 10 years.
+Travel itinerary to Tasmania demonstrated by airline or Spirit of Tasmania tickets showing date of permanent arrival for you and your dependant in Tasmania.
+Evidence of living in Tasmania since permanent arrival for both you and your dependant, demonstrated by rental agreements or a statutory declaration listing all addresses and dates of stay since arrival in Tasmania (which also lists all household tenants).
+Bank statements that show spending on living expenses in Tasmania and any pay or salary deposits since the date you arrived. The statements must be on official bank letter head, clearly showing the account number and account holder's name, and be free of highlighting or any other changes. If your dependant has separate bank statements, you must provide their bank statements that show their living expenses in Tasmania.
+Business bank and personal bank transaction statements for 12 months of most recent operations
+ABN/ASIC certificate.
+Current Company Extract ( https://connectonline.asic.gov.au )
+Business Activity Statements (BAS) for the duration of business operation claimed.
+Australian Taxation Office (ATO) income statement as evidence of personal income claimed from the business. The statement must clearly show your name and have originated from the ATO.
+Business registration and operational evidence as follows:
+Australian Taxation Office annual Notice of Assessment and Lodgement confirmation
+Statement of Distribution if operating as partnership with spouse.
+Photographic evidence of business location and operations.
+Current and previous employment contract and employment confirmation letter signed and dated by the employer outlining pay, conditions and position duties.
+Signed Employer Statutory Declaration form (PDF 754.8 KB)
+Pay slips covering the duration of your employment.
+Australian Taxation Office (ATO) income statement for all employment claims.
+Payslips covering the duration of all employment claims.
+Superannuation Fund transaction statement for the period of any employment you are claiming. The statements must clearly show all employer contributions be on official fund letter head, and clearly show the account number and account holder's name.
+Australian Taxation Office (ATO) income statement for all employment claims.
+Evidence that your pay and conditions are consistent with local market rates. All employment must comply with the Fair Work Ombudsman's National Employment Standards, with pay and conditions no less than those of Australian citizens or permanent residents in comparable roles, and consistent with current local market rates.
+job advertisements from the past six months for comparable positions in the same region on websites such as Seek, Indeed, CareerOne, and either:
+Salary survey data from Hays Guides or SmartMatch ,
+Information from Jobs and Skills Australia's Jobs and Skills Atlas
+Business registration and operational evidence as follows:
+• ABN/ASIC certificate.
+• Current Company Extract ( https://connectonline.asic.gov.au )
+Business bank and personal bank transaction statements for 12 months of most recent operations.
+Business Activity Statements (BAS) for the duration of business operation claimed.
+ATO Income Statement as evidence of personal income claimed from the business.
+Australian Taxation Office annual Notice of Assessment and Lodgement confirmation
+Statement of Distribution if operating as partnership with spouse.
+Photographic evidence of business location and operations.
+ABN/ASIC certificate.
+Current Company Extract ( https://connectonline.asic.gov.au )
+Evidence of sponsoring employer support: If currently holding a Temporary Skill Shortage or Skills in Demand visa (subclass 482) and worked less than 12 months with their Tasmanian-based sponsoring employer.
+Outstanding Tasmanian debts and payment plan summary: This is required if you have an outstanding debt that is signed and witnessed.
+Declaration of nomination obligations: Required if application has been submitted by a Migration Agent.
+Appointment of a registered migration agent legal practitioner or exempt person Form 956 (PDF) : Required if application has been submitted by a Migration Agent.
+Personal statement that is a maximum one-page summary of your current situation and intentions. It is very important to include this where your ties to Tasmania are unclear, you have lived in another part of Australia for a more than 2 years before moving to Tasmania or your family members are overseas or have only recently joined you.
+Include the following points:
+• Why do you want to live in Tasmania?
+• What community support is available to help you settle?
+• What career, business prospects or opportunities do you have in Tasmania?
+• Which family members settling with you. Where are they? When did they arrive in Tasmania? Are they currently studying or working?
+• If your spouse/partner or any dependants are currently overseas, explain why.
+• If they have recently moved to Tasmania from another Australian state or territory, explain what they intend to do in Tasmania.
+Why do you want to live in Tasmania?
+What community support is available to help you settle?
+What career, business prospects or opportunities do you have in Tasmania?
+Which family members settling with you. Where are they? When did they arrive in Tasmania? Are they currently studying or working?
+If your spouse/partner or any dependants are currently overseas, explain why.
+If they have recently moved to Tasmania from another Australian state or territory, explain what they intend to do in Tasmania.
+Tasmanian drivers' license.
+Evidence of job offers and interviews unless previously listed as required
+Adult dependant's passport bio-data page.
+Adult dependant's current resume.
+Dependant child/children passports bio-data pages.
+Adult dependant's skills assessment if available.
+Adult dependant's employment contract if claiming dependant employment priority attributes.
+Evidence of marriage, dependant relationship if claiming to meet dependant-related priority attributes. Adult dependant must be included in Expression of Interest on SkillSelect.</t>
         </is>
       </c>
     </row>

</xml_diff>